<commit_message>
Palmola Health Fisrt Draft
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -1,115 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\documents\docs\me\job\applications\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{149EF79E-5A3E-4AAC-9CC4-9F47A40A48D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{18D3A4F4-489C-4F1C-A2ED-38229FC2BD23}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>ResumeLink</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>IsTaylored</t>
-  </si>
-  <si>
-    <t>JobURL</t>
-  </si>
-  <si>
-    <t>DateApplied</t>
-  </si>
-  <si>
-    <t>DatePosted</t>
-  </si>
-  <si>
-    <t>https://job-boards.eu.greenhouse.io/palomahealthuk/jobs/4939431101?gh_src=flfp2s62teu</t>
-  </si>
-  <si>
-    <t>AI Engineer</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>London</t>
-  </si>
-  <si>
-    <t>Paloma Health</t>
-  </si>
-  <si>
-    <t>RemoteStatus</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -126,27 +52,86 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -466,73 +451,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4635DB4B-305D-4C87-96F0-FC7752495BD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.21875" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="13.5546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="10.21875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.21875" customWidth="1" min="5" max="5"/>
+    <col width="10.77734375" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" t="s">
-        <v>14</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DateApplied</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>JobURL</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ResumeLink</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>IsTaylored</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>DatePosted</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>RemoteStatus</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+    <row r="2">
+      <c r="A2" s="2" t="n">
         <v>46294</v>
       </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" t="s">
-        <v>12</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paloma Health</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Founding AI Engineer on Paloma's AI squad: build and evaluate agentic, LLM-powered applications for NHS children's autism and ADHD assessments, run eval pipelines (gold datasets, prompt/pipeline versioning), and champion evaluation-driven development. Reports to VP Technology.</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/palomahealthuk/jobs/4939431101?gh_src=flfp2s62teu</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>jobs/paloma_health/KaustubhSonawaneAIEngineer.docx (cover letter: jobs/paloma_health/KaustubhSonawaneAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Hybrid (2 days/week London Bridge, Wed/Thu)</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{F59D1522-B122-43D5-A774-BFC5E18B0855}"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Palmola health Applied and Curry's First Draft
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -15,7 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Aptos Narrow"/>
@@ -456,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -569,6 +571,47 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Currys</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AI Engineer (Vacancy ID 50189, Grade 3, permanent) in Tech and Transformation: build AI solutions and agents with product managers across stores, contact centres, trading and supply chain; prototype with LLM/agent frameworks, take features to production, monitor quality, performance and cost. Python, APIs, RAG; Databricks/Azure AI beneficial.</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>jobs/curry's/KaustubhSonawaneAIEngineer.docx (cover letter: jobs/curry's/KaustubhSonawaneAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>London (Waterloo)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Hybrid (in person 2-4 times/month)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
BSC, Moon, Moonpig, Prima, Tank applied
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -15,9 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Aptos Narrow"/>
@@ -56,10 +54,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -612,6 +611,211 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Better Society Capital</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AI Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AI Full Stack Engineer (Investment dept, reports to Head of AI; AI team of two), GBP 50,400-65,800, permanent. AI Innovation Lab work: agentic workflows, prompt/skill library, MCP connectors for Claude, data pipelines with the data team, Technical Design Authority. Python, LLM/RAG/evals, Microsoft ecosystem and Anthropic products desirable. Applied via Applied (anonymised). Closes 11 Oct 2026; no sponsorship offered.</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>jobs/better_society_capital/KaustubhSonawaneAIFullStackEngineer.docx (cover letter: jobs/better_society_capital/KaustubhSonawaneAIFullStackEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>London (EC1Y, Old Street)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Hybrid (40-60% in office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tank Recruitment (client undisclosed)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Data Scientist (Generative AI)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Data Scientist x2 (Ref BBBH97524) for a global data and AI consultancy (insurance, healthcare, banking, retail): lead design and deployment of GenAI solutions - LLM applications, prompt engineering, fine-tuning, embeddings, RAG with vector databases (FAISS, Pinecone, ChromaDB), APIs via FastAPI/Streamlit/Flask; evaluate performance, bias, latency and cost. GBP 80,000-90,000 + bonus. Permanent, immediate start.</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>jobs/tank_requiretment/KaustubhSonawaneDataScientist.docx</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Hybrid (flexible)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Prima</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Software Engineer - Machine Learning</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Software Engineer in Prima's Claims Machine Learning team (motor insurance; 350+ engineers). Software-engineer-first: clean, production-ready Python; Pandas, NumPy, PyTorch/TensorFlow, Hugging Face, GenAI; Postgres; broad ML (classical, deep learning, computer vision, generative AI). Nice to have: international experience, large datasets, Elixir/Rust, AWS. Salary not stated.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>jobs/prima/KaustubhSonawaneMLSoftwareEngineer.docx (cover letter: jobs/prima/KaustubhSonawaneMLSoftwareEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>UK (office location not stated)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Flexible (home, office or mix; work from anywhere up to 30 days/year)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Moon Commerce Limited</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AI Automation Engineer (Agentic Automation Platform)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Hands-on AI automation role (reports to Technology Lead; early-stage UK tech company across commerce, consulting, property, SaaS): build and test agentic workflows using LLM APIs, RAG over internal/client documents, third-party API integrations, write evaluations, take workflows from prototype to unattended production, document. Python 2+ yrs, LLM API, REST/JSON, RAG, Git; nice: vector DBs, LangChain/LlamaIndex, AWS, n8n/Zapier/Make. GBP 35,000-39,000, permanent. Right to work required, no sponsorship. Job title not stated in JD.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>jobs/mooncommerece_limited/KaustubhSonawaneAIAutomationEngineer.docx (cover letter: jobs/mooncommerece_limited/KaustubhSonawaneAIAutomationEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>UK (office area not stated)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Hybrid (2 days/week in office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Moonpig Group</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Applied Data Scientist (hybrid, 1-2 office days/week) building, evaluating and productionising ML for recommendations, personalisation, customer and predictive modelling. Python and SQL, supervised ML and evaluation, A/B test design and analysis, ML pipelines with Engineering/MLOps, monitoring, AI-assisted dev tools. AWS, Git, dbt; LLM/embedding experience useful. Salary: competitive, not stated.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>jobs/moonpig/KaustubhSonawaneDataScientist.docx (cover letter: jobs/moonpig/KaustubhSonawaneDataScientistCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>London or Manchester</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Hybrid (1-2 days/week in office)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
Viridien, Ten Lifestyle Group, SII, Compare The Market
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1132,6 +1132,198 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Viridien</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Forward Deployed AI Engineer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Forward Deployed AI Engineer in Viridien's AI Lab (req JR101453): adapt, integrate and deploy agentic AI, LLM and vision-language systems in production across cloud, on-premises, hybrid and restricted environments; build connectors, APIs and MCP tools, CI/CD and deployment workflows; implement authentication, access control, secrets management and auditability; set up monitoring, logging, tracing, alerting and evaluation; troubleshoot production issues. Needs Python, LLMs/agents/RAG, APIs, Docker, cloud, enterprise security. Desirable: Kubernetes, Helm, Terraform, LangGraph/AutoGen/smolagents, MCP, LLM gateways, AI observability, scientific/geoscience AI. Salary not stated; bonus scheme, 22 days leave.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>jobs/viridien/KaustubhSonawaneForwardDeployedAIEngineer.docx (cover letter: jobs/viridien/KaustubhSonawaneForwardDeployedAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Crawley, UK</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Hybrid (2 days/week at home)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ten Lifestyle Group</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>AI Engineer in Ten's London AI team (lifestyle and concierge services for 50+ clients incl. HSBC, Visa, Mastercard, Amex; B Corp, LSE AIM-listed): design, build, deploy and monitor AI systems at scale in a cross-functional 'you build it, you run it' DevOps team; automated testing and metrics; weigh cost and timelines. Needs a programming language, Gen AI tools (LangGraph, CrewAI, Hugging Face, OpenAI APIs), ML fundamentals and LLM challenges (latency, cost, hallucinations, evaluation), cloud and IaC (Terraform), CI/CD, Docker, K8s, observability (Prometheus, Grafana, Datadog), distributed systems, SQL and NoSQL; agents and multi-agent workflows desired. Salary: competitive, not stated; 25 days leave, pension.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>jobs/ten_lifestyle_group/KaustubhSonawaneAIEngineer.docx (cover letter: jobs/ten_lifestyle_group/KaustubhSonawaneAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Hybrid (at least 2-3 days/week in office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Compare the Market</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer in Compare the Market's Data &amp; AI Solutions function: take ML models and AI capabilities from experimentation to reliable, scalable production (pipelines, deployment tooling, monitoring, shared components); package, deploy and automate model lifecycle; monitor performance, drift and reliability; support batch and real-time workloads; integrate LLM-powered capabilities; promote CI/CD, reproducibility, testing, model and agent observability and evaluation; work with data scientists to productionise prototypes; responsible AI (explainability, auditability, fairness). Essentials: production/near-production ML or AI components, Python, Databricks/MLflow/Airflow or equivalent, CI/CD for ML, ML lifecycle (versioning, testing, monitoring, governance). Nice to have: LLM/RAG/LangGraph/LangChain, multi-step agents, agentic coding tools, regulated sector. Salary not stated.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>jobs/compare_the_market/KaustubhSonawaneMLEngineer.docx (cover letter: jobs/compare_the_market/KaustubhSonawaneMLEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Hybrid (London office)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SII UK (SII Group)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>AI Engineer for Autonomy</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>AI Engineer for Autonomy at SII UK, Aerospace &amp; Defence engineering partner (permanent): design, develop and deliver AI/ML for safety-critical defence programmes across computer vision, autonomy, LLMs and predictive analytics; data processing, training and evaluation pipelines; Responsible AI (robustness, explainability, security); deploy to production with software engineers; model performance and drift monitoring; reusable AI components; customer demos, PoCs and bids. Essential: strong Python, PyTorch/TensorFlow/Scikit-Learn, ROS2 or equivalent, CV/DL/NLP/LLM/time-series, Pandas/NumPy/SQL, Git/CI, Agile, DevOps/MLOps, eligible for UK Security Clearance (SC). Desirable: MLflow/W&amp;B, Spark, ONNX/TorchScript/FastAPI/gRPC, cloud, Docker, C++ in safety-critical environments. Salary not stated.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>jobs/sii_group/KaustubhSonawaneAIEngineerAutonomy.docx (cover letter: jobs/sii_group/KaustubhSonawaneAIEngineerAutonomyCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>UK (Belfast, Chester, Farnborough, London or Oxford; office not specified)</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
ByteIO mailed, Halfords not able to apply. Contact Hiring Manager.
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1324,6 +1324,57 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Byte</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>AI Engineer at Byte (London, full-time, hybrid): work directly with the CTO on a personal AI agent for students; build retrieval pipelines, structured model outputs and tool-execution workflows; Outlook/calendar integrations (OAuth, webhooks, background jobs, sync); personal memory with source references and access controls; own backend, database and React frontend; reliable actions (idempotency, retries, approvals); evaluation datasets; tests, deployment and instrumentation. Needs strong Python and SQL, LLM apps with retrieval/structured outputs/tools, ML fundamentals, transformers, API/auth/queues/concurrency, TypeScript and React. Useful: PostgreSQL, vector search, Redis, Docker, CI/CD, Microsoft Graph, agent frameworks. Apply by email to jeffrey@usebyte.io (CV plus links to work); process includes a ~90-minute online assessment. Salary not stated.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Email: jeffrey@usebyte.io (no application portal)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>jobs/byte_io/KaustubhSonawaneAIEngineer.docx (cover letter / email body: jobs/byte_io/KaustubhSonawaneAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Email To Send</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
UBE, Apexon, Gazette Global, La Fosse
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1491,6 +1491,276 @@
         <v>1</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>University of the Built Environment (UBE)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Software Engineer (Python and AI Solutions)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Software Engineer (Python and AI Solutions) in UBE's COO Technology team, Reading (permanent, full time, 35 hrs/week; line manager Tony Phillips, Solutions Architecture and Development Manager; closes Mon 26 Oct 2026 17:00): design, develop, test, deploy and maintain Python applications, APIs, integrations and backend services; design AI-enabled solutions, evaluate and integrate generative AI incl. Microsoft Copilot, build AI-powered workflows and automation, align with AI governance, security and privacy; secure coding, code reviews, UAT, automated test suites in CI/CD, documentation, performance monitoring. Essential: degree in CS/IS or equivalent experience, enterprise software, AI/LLM solutions, Python, APIs and integrations, cloud (Azure preferred), source control, automated testing and CI/CD, security, data protection and accessibility. Salary £40,000-£45,000. Informal contact: Emma Stone, e.stone@ube.ac.uk.</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>https://ube-careers.teamtailor.com/jobs/8551684-software-engineer-python-and-ai-solutions</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>jobs/ube/KaustubhSonawaneSoftwareEngineer.docx (cover letter: jobs/ube/KaustubhSonawaneSoftwareEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Horizons, Reading, UK</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Hybrid (minimum 2 days/week at Horizons)</t>
+        </is>
+      </c>
+      <c r="L21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Apexon</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>AI Engineer at Apexon (Bengaluru; AI-first technology services firm backed by Goldman Sachs Asset Management and Everstone Capital; 5-8 years experience asked): build enterprise-grade GenAI and agentic AI workflows for financial-services exception classification, triage, root-cause analysis, impact assessment and remediation across large transaction and data-processing environments; agentic workflows with orchestration, tool/function calling, state management and human-in-the-loop validation; Python and SQL services over structured enterprise data; FastAPI backends and enterprise API/ticketing integrations; RAG over regulatory documents and issue repositories; confidence scoring, validation, guardrails and traceability; testing, logging, evaluation and observability. Needs hands-on LangGraph, Google ADK, CrewAI, AutoGen, Semantic Kernel or a custom orchestration framework. Nice to have: MCP, knowledge graph/Graph RAG, vector DBs and re-ranking, AI observability and evaluation, spec-driven development, Claude Code, basic React. Preferred domain: regulatory reporting, capital markets, EMIR/MiFID II/SFTR. Salary not stated.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs-india/apexon/JDAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>jobs-india/apexon/KaustubhSonawaneAIEngineer.docx (cover letter: jobs-india/apexon/KaustubhSonawaneAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gazelle Global</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>AI Engineer on an enterprise AI platform programme (recruiter posting from Gazelle Global; end client not named): turn platform services into practical AI-driven business capabilities across enterprise applications, workflows and SDLC; build RAG pipelines and knowledge retrieval workflows, design prompt strategies and guardrails, configure agent workflows and reusable orchestration patterns, work with SMEs to refine domain behaviour, run structured evaluation and iteratively improve, contribute reusable AI patterns to the platform. Key skills: hands-on LLM API, production RAG or agent systems, strong API and integration skills, prompt engineering and guardrails, AI evaluation and hallucination mitigation, Responsible AI, agent orchestration. Apply by email Mir@gazellegc.com. Salary not stated. (JD jobs/gazelle-global/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Email: Mir@gazellegc.com (no application portal)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>jobs/gazelle-global/KaustubhSonawaneAIEngineer.docx (cover letter / email body: jobs/gazelle-global/KaustubhSonawaneAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="L23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Lafosse</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BI Engineer</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BI Engineer (permanent, full-time, circa £60K; recruiter posting by Lafosse, end client in the transportation sector not named) reporting to the Lead BI Engineer: build and maintain ETL/ELT pipelines and reporting datasets; SQL and Python (incl. PySpark) transformations; monitor and tune pipelines and queries; data quality controls and documentation; translate business requirements into data solutions; support BI developers, dashboards and self-service analytics adoption; incident management. Needs AWS data services (Redshift, Athena, S3, Glue, Lambda), strong SQL, Python/PySpark, Git/CodeCommit, stakeholder engagement. Nice to have: SnapLogic or similar, open table formats, DuckDB, QuickSight/Power BI/Tableau. (JD jobs/lafosse/JDBIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/lafosse/JDBIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>jobs/lafosse/KaustubhSonawaneBIEngineer.docx (cover letter: jobs/lafosse/KaustubhSonawaneBIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Hybrid (3 days/week onsite)</t>
+        </is>
+      </c>
+      <c r="L24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lafosse</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Power BI Engineer (Contract)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Power BI Engineer contract via recruiter Lafosse (end client not named; inside IR35, 550-600 GBP/day, initial 6 months, Central London 2 days/week onsite): hands-on Power BI development on a major global reporting programme, building reports from established designs and templates; interactive multi-page reports, semantic models and datasets, DAX measures, Power Query; connect Power BI to Databricks and other enterprise sources; work with Data Engineers, Product Owners and stakeholders. Required: Power BI, DAX, semantic modelling, Power Query, Databricks, SQL, data visualisation. Desirable: Azure Databricks/Lakehouse, Power BI Service, deployment pipelines/DevOps, large-scale enterprise reporting, Microsoft Fabric. Apply directly via Lafosse. (JD jobs/lafosse/JDPowerBIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/lafosse/JDPowerBIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>jobs/lafosse/KaustubhSonawanePowerBIEngineer.docx (cover letter: jobs/lafosse/KaustubhSonawanePowerBIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>To Apply</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Central London</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Hybrid (2 days/week onsite)</t>
+        </is>
+      </c>
+      <c r="L25" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
Saragossa, Capsa, Callosum, LinuxRecruit, IntelStack
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Security Clearance Required</t>
+          <t>Security Clearance Required Thus Not Applied</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1866,6 +1866,276 @@
         </is>
       </c>
       <c r="L27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Saragossa (recruiter; AI consultancy client not named)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>AI Engineer (Python-led)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>AI Engineer (Python-led), permanent, up to GBP 140,000 base + equity, London relocation; posted by Saragossa, a talent/technology recruiter for investment businesses, on behalf of an unnamed fast-growing AI consultancy. No formal job posting: applied by LinkedIn cold DM to the poster plus the 'Work for us' form on saragossa.io (specialism AI, Permanent UK). Role: build LLM/GenAI client solutions with a team of AI Engineers, owning the Python/backend side (great Python developer, data and microservices experience a plus, some LLM/GenAI experience, not expert); liaise with clients; hybrid with travel to client sites. 'No up-to-date CV required.' Reserve CV (software-engineer framing) held back in case the client wants a backend-first profile. (JD jobs/saragossa/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>https://saragossa.io/contact/ (LinkedIn cold DM to poster; no job posting URL)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>jobs/saragossa/KaustubhSonawaneAIEngineer.docx + .pdf (DM and form text: jobs/saragossa/KaustubhSonawaneAIEngineerCoverLetter.docx; reserve CV: jobs/saragossa/KaustubhSonawaneSoftwareEngineer.docx + .pdf)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>London (relocation)</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Hybrid (travel to client sites); up to GBP 140k + equity</t>
+        </is>
+      </c>
+      <c r="L28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Capsa</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Senior AI Engineer in Capsa's engineering team (AI Operating System for private capital funds; Series A, ARR up 15x), London, hybrid with 4 days a week in person; competitive base + ESOP. Build and own the agent harness (custom streaming-first graph execution framework), a resumable code execution framework for programmatic tool calling, VLM-based OCR document ingestion with a self-hosted search cluster (OpenSearch), citations for every AI-generated claim, and document authoring across Word, Excel, PowerPoint and email; own agent capabilities end to end, from harness internals to evals. Required: 5+ years building production backend systems at a venture-backed startup or top tech firm owning AI-powered services; agents, retrieval or LLM features shipped to production with eval results; Python, LLMs, agents, retrieval and search (OpenSearch), evals, FastAPI, Postgres, RabbitMQ; TypeScript and React a plus. (JD jobs/capsa/JDSeniorAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/capsa/JDSeniorAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>jobs/capsa/KaustubhSonawaneSeniorAIEngineer.docx + .pdf (cover letter: jobs/capsa/KaustubhSonawaneSeniorAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Hybrid (in person 4 days/week)</t>
+        </is>
+      </c>
+      <c r="L29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Linux Recruit (unnamed enterprise AI platform startup)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Full Stack AI Engineer</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Full-stack AI engineer at an unnamed, well-funded (GBP 70m+ raised) enterprise AI operating platform startup, advertised by recruiter Linux Recruit (Ethan Farrell); small team, ships in days across the full stack, customer-facing alongside founders; Kotlin, TypeScript, Python; builder's DNA (side projects, startups, open source); shipped AI products in production; product intuition; excellent compensation, equity and full visa sponsorship if required. Required (poster): Bachelor's degree, 2+ years agentic AI development, 2+ years LLMs. Applied via LinkedIn Easy Apply plus an email to the recruiter. (JD jobs/linuxrecruit/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply + email ethan.farrell@linuxrecruit.co.uk (no job URL; JD saved in jobs/linuxrecruit/JD.txt)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>jobs/linuxrecruit/KaustubhSonawaneFullStackAIEngineer.docx + .pdf (recruiter email and Easy Apply note: jobs/linuxrecruit/KaustubhSonawaneFullStackAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Not stated (UK)</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="L30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Callosum</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer (Member of Technical Staff)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer on Callosum's Applied AI team (Member of Technical Staff structure; $100M round led by Atomico; builds the software orchestration layer for heterogeneous compute: Cerebras, d-Matrix, NVIDIA, AMD, Tenstorrent and others), London, in person; competitive salary (not stated) + equity, private healthcare, visa sponsorship and relocation offered. Own customer engagements end to end: scope customer AI workloads (retrieval pipelines, agentic workflows, code intelligence stacks), design and run rigorous evaluations on production pipelines, integrate optimised workflows into customer environments and support them into production, feed learnings to research and platform teams, build the team's evaluation harnesses, integration runbooks and engagement standards. Needs technical depth (production systems at scale, shipped research or founding role), experience with LLM serving infrastructure, agent orchestration or retrieval systems, rigour in evaluation or benchmarking, bias for action; plus: forward deployed engineer / solutions architect experience, novel accelerator platforms, early-stage or founding-engineer role. (JD jobs/callosum/JDAppliedAITechnicalStaff.txt)</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/callosum/JDAppliedAITechnicalStaff.txt)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>jobs/callosum/KaustubhSonawaneAppliedAIEngineer.docx + .pdf (cover letter: jobs/callosum/KaustubhSonawaneAppliedAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>On-site (in person at London office)</t>
+        </is>
+      </c>
+      <c r="L31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Intelstack</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>AI Engineer (12-month contract)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>AI Engineer on a 12-month contract (Inside IR35) at Intelstack, London, hybrid 3 days a week (day rate not stated): design, develop and deploy AI-powered applications using LLMs and Generative AI; build engineering solutions with GitHub Copilot, Claude Code, OpenAI, Azure OpenAI and Anthropic Claude; develop AI agents, copilots and workflow automation for enterprise use cases; RAG solutions over vector databases; prompt engineering frameworks and evaluation mechanisms; integrate AI services with enterprise applications via APIs, microservices and cloud-native architectures; build automated coding assistants and developer productivity tools; AI governance, security, model monitoring and responsible AI; mentor development teams on AI-assisted development tools. Essential: strong LLM and Generative AI experience. Desirable: Azure/AWS/GCP, CI/CD (GitHub Actions, Azure DevOps, Jenkins), Docker and Kubernetes, Infrastructure as Code (Terraform preferred). (JD jobs/intelstack/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/intelstack/JD.txt)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>jobs/intelstack/KaustubhSonawaneAIEngineer.docx + .pdf (cover letter: jobs/intelstack/KaustubhSonawaneAIEngineerCoverLetter.docx)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Hybrid (3 days/week); 12-month contract, Inside IR35</t>
+        </is>
+      </c>
+      <c r="L32" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Angstrom Sports, IMC, G-Research
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2812,6 +2812,222 @@
         <v>0</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>G-Research</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer in the ML and HPC Architecture team at G-Research (London HQ; quantitative finance; highly competitive compensation plus annual discretionary bonus and 9% company pension). Identify and work with tools at the cutting edge of machine learning, collaborating with Quant Researchers, Quant ML engineers, other engineering groups, external partners and vendors. Past projects: evaluating alternative accelerators for ML workloads; multi-node distributed training to understand trade-offs in networking technology; optimising model inference to minimise latency or maximise throughput; understanding and optimising storage technology to maximise bandwidth; evaluating the latest hardware and software in the ML ecosystem; liaising with vendors and giving constructive feedback on their products and roadmaps. Ideal candidate: a postgraduate degree in ML or a related field, or commercial experience building ML models at scale, or demonstrable success in online data-science competitions such as Kaggle; strong object-oriented engineering with Python (PyTorch and NumPy desirable); the ability to apply advanced optimisation methods, modern ML techniques, HPC, profiling or model-inference expertise (not all required); a passion for the latest ML and HPC trends; excellent communication and the ability to present results to stakeholders; choosing the right level of abstraction, from quick proof-of-concept scripts to complex systems. Finance experience is not necessary. (JD: jobs/gresearch/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/gresearch/JD.txt)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>jobs/gresearch/KaustubhSonawaneMLEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="n"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Not stated in JD (JD lists Location: London only)</t>
+        </is>
+      </c>
+      <c r="M45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>IMC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer (Technology, London) at IMC, a research-driven trading firm; brand new position in a growing team. Build systems for training and deployment of large-scale ML models: distributed training pipelines for large datasets and complex models; low-latency inference pipelines delivering real-time predictions in production; libraries to improve ML framework performance; maximise training and inference performance on GPU hardware and acceleration libraries; scalable model frameworks for high-volume trading data; automate ML experiments, hyperparameter tuning and retraining with quantitative researchers; partner with HPC specialists on training speed and cost; evaluate third-party tools; dig into open-source ML tool internals. Required: 5+ years in machine learning focused on training or inference systems; strong engineering in Python, CUDA or C++; PyTorch, TensorFlow or JAX; GPU programming (cuDNN, TensorRT); distributed training (Horovod, NCCL); cloud platforms and orchestration tools. Plus: real-time low-latency ML pipelines, open-source contributions. (JD: jobs/imc/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/imc/JD.txt)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>jobs/imc/KaustubhSonawaneMLEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="n"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Not stated in JD (JD lists London only)</t>
+        </is>
+      </c>
+      <c r="M46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Angstrom Sports (Entain)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Data Science Manager</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Data Science Manager, Data &amp; Analytics department at Angstrom Sports (Entain group; proprietary sports pricing, player-level play-by-play simulation-driven pricing and risk systems, US sports-first). Hybrid, London or Leeds office, full-time. Manage Data Science Leads and grow high-performing teams; align delivery across multiple projects, sports and technical domains; set and maintain modelling standards, code practices and documentation; address capacity, capability and performance challenges; work with Delivery Engineering and the Head of Data Science on strategy, tooling and hiring plans; escalation point for technical resourcing; represent Data Science in leadership meetings. Essential: demonstrated success managing Data Science Leads (2+ years managing teams); strong technical background in model development and deployment; advanced programming (R/Python/C#/Java); hiring, performance and team development; sports modelling and betting domain expertise. Desirable: scaling data science functions, model governance/risk/compliance, tooling and infrastructure, AWS, STEM degree. (JD: jobs/angstromsports/JDDataScienceManager.txt)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/angstromsports/JDDataScienceManager.txt)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>jobs/angstromsports/KaustubhSonawaneDataScienceManager.docx + .pdf (cover letter is a message box in the application form: jobs/angstromsports/KaustubhSonawaneDataScienceManagerMessage.txt)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="n"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>London or Leeds</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Hybrid (London or Leeds office)</t>
+        </is>
+      </c>
+      <c r="M47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Angstrom Sports (Entain)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Data Engineer, Data &amp; Analytics department at Angstrom Sports (Entain group; proprietary sports pricing, player-level play-by-play simulation-driven pricing and risk systems, US sports-first). Hybrid, London or Leeds office, full-time. Salary GBP 45,000-65,000. Design and implement scalable data architectures; build and maintain ETL pipelines; manage data storage, backup and recovery; write SQL for analysis; data security and privacy; interface with clients and end users. Essential: clean SQL and Python for transformation/analytics; data modelling; 2+ yrs relational databases; 1+ yr pipelines on Kafka or equivalent event streaming; debug/optimise slow pipelines and queries; systems integration (networking, migrations, API design); 2+ yrs AWS S3, Athena, ECS, CloudFormation, Lambda, CloudWatch; documentation, logging, reproducibility. Desirable: Power BI/Superset, Spark/Kafka, TDD, love of sports, side project showing end-to-end solution architecture. (JD: jobs/angstromsports/JDDataEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/angstromsports/JDDataEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>jobs/angstromsports/KaustubhSonawaneDataEngineer.docx + .pdf (cover letter message box in application form: jobs/angstromsports/KaustubhSonawaneDataEngineerMessage.txt)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>London or Leeds</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Hybrid (London or Leeds office)</t>
+        </is>
+      </c>
+      <c r="M48" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
Apple, ATG, Bioptix, HeartlyCo, Metcor, Softweb Resourcing, SolveIntelligence,Labour Party
</commit_message>
<xml_diff>
--- a/ApplicationTracker.xlsx
+++ b/ApplicationTracker.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3244,6 +3244,550 @@
         <v>0</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Metcor Group</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff - AI Engineer</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Member of Technical Staff - AI Engineer at Metcor Group (UK facilities management, 600+ people), second person in the AI team, reporting to Head of AI Engineering; permanent, full time, GBP 120k, no visa sponsorship (right to work in the UK required). Re-shape how engineering work gets done: job scheduling, predicting and preventing outages, KPIs defined before building. Problems: computer vision on site captures, offline LLMs, agentic-first UX for field engineers, model training and trend spotting on decades of data, geo-routing and scheduling. Essential: agentic systems deployed in production (or a running side project), commercial instincts, knowing where AI beats a rule or query, self-led. Set apart: Lead/Staff level, deep production Python and SQL, own services on a cloud platform, startup background, MSc in Computer Science or related. Apply with CV plus a short note on one agentic thing built, what it was meant to move and whether it did, to janosch.oppermann@metcor.co.uk (no agencies). (JD: jobs/metcor/JDAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/metcor/JDAIEngineer.txt; apply by email to janosch.oppermann@metcor.co.uk)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>jobs/metcor/KaustubhSonawaneAIEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="n"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Hybrid (3 days on site, occasional travel)</t>
+        </is>
+      </c>
+      <c r="M53" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bioptix</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer in the R&amp;D team at Bioptix Ltd (neuroscience technology, founded 2021), reporting to the Technical Director; salary GBP 60-80k. Leads development, training and improvement of the AI agent that operates the automated experimental platform, and owns the training strategy: agent design (imitation learning, reinforcement learning, supervised policy learning or hybrid rule-and-model), action and observation spaces, training/fine-tuning/deployment pipelines with versioning and reproducibility, integration with real-time control software, sensors and instrument hardware, simulation or offline test environments; specifying data needs, collection protocols, labelling, QC and versioning pipelines; evaluation metrics and benchmark suites, failure diagnosis, drift detection and retraining, documentation for a regulated product environment. Required: degree in CS/ML/Engineering/Maths/Physics (poster adds Master's and 1+ years research), production ML, Python plus PyTorch/TensorFlow/JAX, end-to-end training pipelines, specifying data requirements, diagnosing model failure, working with domain experts. Desirable: neural-network and maths depth, agentic/RL/imitation learning, ML on physical systems or lab automation, computer vision for microscopy, small-data learning, MLOps experiment tracking, start-up/scale-up, life science instrumentation. (JD: jobs/bioptix/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/bioptix/JD.txt)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>jobs/bioptix/KaustubhSonawaneMachineLearningEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="n"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="M54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Heartly &amp; Co (recruiter; employer unnamed)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Founding AI Engineer</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Founding AI Engineer (employee #3) at an unnamed early-stage London AI-first product studio (recruiter-posted), GBP 100-150k + equity, in-person, working directly with the founder; well funded, multi-million-dollar round from technology and gaming investors. Builds agent systems that turn a spec into a shipped, live product. Own the agent process (model selection, prompting, agent loop/orchestration design) and the context layer (managing context, using data to improve agent output); extend the current agent pipeline for deeper context and planning; shape AI use across the whole product. Wants: someone who has built AI agents that write, test or ship code (not just Q&amp;A or business-task agents); hands-on builder energy with heavy personal use of Claude Code or Cursor, side projects, hackathons or open source; comfortable in an early-stage, in-person, high-ownership environment. Right to work in the UK required. (JD: jobs/heartlyco/JDFoundingAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/heartlyco/JDFoundingAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>jobs/heartlyco/KaustubhSonawaneFoundingAIEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="n"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>On-site (in person)</t>
+        </is>
+      </c>
+      <c r="M55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Solve Intelligence</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>AI Engineer at Solve Intelligence (Series B legal-AI/IP startup, ~$55M backing, London team; full visa sponsorship offered). Build and improve production AI agents for drafting, analysing and evaluating patents; own context management, tools and prompt engineering (with IP experts) so agents handle thousands of documents reliably; build a state-of-the-art evaluation pipeline benchmarking performance across large datasets. Essential: expert Python, industry experience shipping agents and/or evaluation pipelines to production, context and prompt engineering, back-end and Postgres, front-end TypeScript/React, clear writing. Nice to have: publications at top ML conferences. Salary not stated. (JD: jobs/solveintelligence/JDAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/solveintelligence/JDAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>jobs/solveintelligence/KaustubhSonawaneAIEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Not stated (London team)</t>
+        </is>
+      </c>
+      <c r="M56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Softweb Resourcing (recruiter; employer unnamed)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Graduate C++ Software Engineer - Computer Vision</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Graduate C++ Software Engineer - Computer Vision at Softweb Resourcing (recruiter-posted; end employer unnamed): graduate role building C++ systems for real-time media and video environments, with training and mentoring; hybrid/flexible; competitive salary and bonus (not stated). Required: knowledge of C++ and Python through coursework, projects or a dissertation; understanding of computer vision, video / image processing; problem-solving; communication; 2.1+ Bachelors, Master or PhD in a STEM subject. Beneficial: GPU / CUDA / OpenCL, video performance. R&amp;D-minded, geospatial / video / image-processing exposure welcome. (JD: jobs/softwebresourcing/JDGraduateSoftwareEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/softwebresourcing/JDGraduateSoftwareEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>jobs/softwebresourcing/KaustubhSonawaneGraduateSoftwareEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Wrong CV Submitted</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="n"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Hybrid / flexible</t>
+        </is>
+      </c>
+      <c r="M57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Softweb Resourcing (recruiter; employer unnamed)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Software Engineer (C++, Python, React)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Mid-Level Software Engineer (C++) at an unnamed ethical fintech (recruiter-posted via Softweb Resourcing), fully remote UK, up to GBP 65k base, flexible hours. Develop and maintain modern C++; build Python microservices and tooling; React/TypeScript frontends; AWS, Docker, CI/CD and Infrastructure as Code; support deployment and scaling of AI/ML services; write tested, secure code. Required: strong commercial C++ 17/20/23, Python, AWS/cloud, REST APIs, microservices and CMake, Git/testing/Linux, Cursor and/or Claude Code. Desirable: Open Banking, fintech/payments, React, OAuth2/OIDC, DynamoDB. UK work authorisation required. (JD: jobs/softwebresourcing/JDSoftwareEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/softwebresourcing/JDSoftwareEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>jobs/softwebresourcing/KaustubhSonawaneSoftwareEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>UK (remote)</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Fully remote</t>
+        </is>
+      </c>
+      <c r="M58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Softweb Resourcing (recruiter; employer unnamed)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Founding AI Engineer (Applied AI / Computer Vision)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Founding AI Engineer (Applied AI / Computer Vision) at an unnamed pre-seed video / computer vision startup (recruiter-posted via Softweb Resourcing), London, hybrid (1 day a fortnight in London), GBP 100-150k base + equity. First dedicated AI hire working directly with the founders; owns AI engineering end to end across product quality, infrastructure efficiency and technical direction; agentic workflows and AI video tools for large-scale media, frontier models already in production, multiple deals signed. Wants: 5+ years in Applied AI / ML / MLOps, experience building eval frameworks, strong Python and production AI systems, LLMs / GenAI / prompt engineering / agentic workflows, startup mindset. Beneficial: computer vision / video / VFX / rendering / graphics. (JD: jobs/softwebresourcing/JDFoundingAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/softwebresourcing/JDFoundingAIEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>jobs/softwebresourcing/KaustubhSonawaneFoundingAIEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Hybrid (1 day a fortnight in London)</t>
+        </is>
+      </c>
+      <c r="M59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>The Labour Party</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Data Scientist</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Data Scientist at The Labour Party (UK - Head Office London, open to flexible or other locations; 1 year fixed-term contract; GBP 50,913.46 gross plus GBP 1,195 fixed-sum allowance, plus GBP 3,760 if London-based; applications close 18 Oct 2026; office four days a week Mon-Thu, home working Fridays only; the application needs a CV and a cover note against the person specification). Conduct polling, advanced modelling and voter targeting, and analyse public opinion, voting behaviour and campaign performance to inform Labour's political and organisational strategies. Essential: strong understanding of statistical modelling (degree-level statistics or equivalent professional experience); strong understanding of polling methodology and how to use polling to answer political questions; experience analysing and reporting on political data and polling, with reports, visualisations and dashboards for stakeholders; ability to see how voter, campaign and election data can drive strategic decisions. (JD: jobs/thelabourparty/JDDataScientist.txt)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/thelabourparty/JDDataScientist.txt)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>jobs/thelabourparty/KaustubhSonawaneDataScientist.docx + .pdf (cover note text for the portal's cover letter box: jobs/thelabourparty/KaustubhSonawaneDataScientistCoverLetter.txt)</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Office-based (4 days a week Mon-Thu, home working Fridays only)</t>
+        </is>
+      </c>
+      <c r="M60" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Data Scientist - WPC - Analytics</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Data Scientist - WPC - Analytics at Apple (London, England; Machine Learning and AI team; Role Number 200685662-2114; posted 15 Oct 2026), in the Wallet, Payments &amp; Commerce Analytics organisation for the Apple Pay business. Strategic analytics partner to senior business leaders across functions: translate complex business questions into structured analytical approaches, apply statistical and advanced analytical techniques to evaluate performance and find growth and efficiency opportunities, deliver data-backed recommendations, and work with data engineering on data quality. Minimum: proven Analytics and Strategy role; strong business acumen; excellent communication (consulting or customer-facing, fast-paced background); SQL, R or Python plus a data visualisation tool such as Tableau; applied statistical/ML techniques. Preferred: Financial Services or Fintech, cross-functional work, handling ambiguous problems, ownership. (JD: jobs/apple/JD.txt)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/apple/JD.txt)</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>jobs/apple/KaustubhSonawaneDataScientist.docx + .pdf (cover letter: jobs/apple/KaustubhSonawaneDataScientistCoverLetter.docx + .pdf)</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="M61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>ATG Entertainment</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer in ATG's small, growing ML team (UK theatre group; Snowflake and AWS data platform). Own defined parts of the revenue management application used across UK, USA and Europe (regional pipelines, seat map and pricing data pulls, model inference): productionise and automate ML models end to end (ingestion, feature engineering, training, evaluation, inference, pricing recommendations); build data pipelines and MLOps workflows (CI/CD, model versioning, reproducibility) in AWS and Snowflake; triage failed pipeline runs and data quality problems; monitor model outputs (data and prediction drift, anomaly detection) with daily dashboards; implement guardrails for pricing recommendations (thresholds, overrides, fallbacks); well-tested Python and SQL with peer review; help design LLM-powered internal tools with prompt management, versioning and evaluation; propensity models and audience segmentation. Essential: ML engineer or data scientist delivering to production, AWS data science workloads, strong Python and SQL, MLOps, monitoring/alerting/observability, reliability concepts (retries, idempotency, fault tolerance), stakeholder communication. Desirable: pricing, revenue optimisation or demand forecasting, monitoring dashboards (Streamlit, BI), LLMs in production, Snowflake, Terraform or SageMaker pipelines. Salary not stated. (JD: jobs/atg/JDMLEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Not provided (JD saved in jobs/atg/JDMLEngineer.txt)</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>jobs/atg/KaustubhSonawaneMLEngineer.docx + .pdf (CV only, no cover letter drafted)</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Awaiting Reply</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="n"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Not stated (UK)</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="M62" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>